<commit_message>
Continue collection: CA/NY/FL/TX page 4-5 and GA/OH/PA/WA/VA/MA/AZ/CO page 2 batches (224 unique firms)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cornell_ip_scraper/output/IP_Law_Firms.xlsx
+++ b/cornell_ip_scraper/output/IP_Law_Firms.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IP Law Firms" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$225</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'IP Law Firms'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B199"/>
+  <dimension ref="A1:B225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -2862,8 +2862,320 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Camuti Law Group APC</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>https://www.camutilaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>Leason Ellis</t>
+        </is>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>http://www.leasonellis.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Chiara IP Law PLLC</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chiaraiplaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>The Lomnitzer Law Firm, P.A.</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>https://www.lomnitzerlaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>Kennedy Law, LLP</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>https://www.saklaw.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="4" t="inlineStr">
+        <is>
+          <t>Grant's Law Firm</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>http://www.grants-law.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>Burgoyne Law Group</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>http://www.burgoynelawgroup.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="4" t="inlineStr">
+        <is>
+          <t>James Hsui, PLLC</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jameshsuilaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>Peppercorn Partners LLC</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>https://www.peppercornpartners.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="4" t="inlineStr">
+        <is>
+          <t>Widerman Malek, PL</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>http://www.legalteamusa.net/daniel-c-pierron-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>Old City Law</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oldcitylaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>Bradley Arant Boult Cummings LLP</t>
+        </is>
+      </c>
+      <c r="B211" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bradley.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>McGurk Intellectual Property Advisors</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>http://www.mcgurkip.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>Briggs Intellectual Property Law</t>
+        </is>
+      </c>
+      <c r="B213" s="5" t="inlineStr">
+        <is>
+          <t>https://www.briggsip.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>Kent &amp; Risley LLC</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kentrisley.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>Cozza Law Group PLLC</t>
+        </is>
+      </c>
+      <c r="B215" s="5" t="inlineStr">
+        <is>
+          <t>http://www.cozzalaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>Elman Technology Law, P.C.</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>https://elman.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="4" t="inlineStr">
+        <is>
+          <t>Claiborne Patent Law Services</t>
+        </is>
+      </c>
+      <c r="B217" s="5" t="inlineStr">
+        <is>
+          <t>http://www.claibornepatent.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>Law Office of Mark B. Saku PLLC</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>http://www.marksakulaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>Keefe IP Law, PLLC</t>
+        </is>
+      </c>
+      <c r="B219" s="5" t="inlineStr">
+        <is>
+          <t>https://www.keefeip.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>Franco Patent Law</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>https://www.francopatentlaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>Mostyn IP, LLC</t>
+        </is>
+      </c>
+      <c r="B221" s="5" t="inlineStr">
+        <is>
+          <t>http://www.mostynip.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>Jaburg Wilk</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>http://www.jaburgwilk.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>Booth Udall Fuller, PLC</t>
+        </is>
+      </c>
+      <c r="B223" s="5" t="inlineStr">
+        <is>
+          <t>https://www.boothudall.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>Hunziker Legal Services, PLLC</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>https://hunzikerlegalservices.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="4" t="inlineStr">
+        <is>
+          <t>Cochran Freund &amp; Young LLC</t>
+        </is>
+      </c>
+      <c r="B225" s="5" t="inlineStr">
+        <is>
+          <t>https://www.patentlegal.com/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B199"/>
+  <autoFilter ref="A1:B225"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -3062,6 +3374,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B197" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B198" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B199" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B200" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B201" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B202" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B203" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B204" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B205" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B206" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B207" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B208" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B209" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B210" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B211" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B212" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B213" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B214" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B215" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B216" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B217" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B218" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B219" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B220" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B221" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B222" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B223" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B224" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B225" r:id="rId223"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToWidth="1"/>

</xml_diff>

<commit_message>
Continue collection: NC/IL/NJ/TN and MD/MN/MO/OR page 2 batches (238 unique firms)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cornell_ip_scraper/output/IP_Law_Firms.xlsx
+++ b/cornell_ip_scraper/output/IP_Law_Firms.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IP Law Firms" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$225</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$239</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'IP Law Firms'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B225"/>
+  <dimension ref="A1:B239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -3174,8 +3174,176 @@
         </is>
       </c>
     </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>Spilman Thomas &amp; Battle, PLLC</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>http://www.spilmanlaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>Morningstar Law Group</t>
+        </is>
+      </c>
+      <c r="B227" s="5" t="inlineStr">
+        <is>
+          <t>http://morningstarlawgroup.com/author/john-kivus/</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>Odin Law and Media</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>http://odinlaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t>Incubate IP</t>
+        </is>
+      </c>
+      <c r="B229" s="5" t="inlineStr">
+        <is>
+          <t>https://www.incubateip.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>Bea &amp; Mays</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>https://bealaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="4" t="inlineStr">
+        <is>
+          <t>Sleman &amp; Lund LLP</t>
+        </is>
+      </c>
+      <c r="B231" s="5" t="inlineStr">
+        <is>
+          <t>http://www.patentspace.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>McNeely, Hare &amp; War, LLP</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>http://www.patentek.com/attorneys/dr-sarika-singh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>Jonathan C Weetman, Attorney at Law, LLC</t>
+        </is>
+      </c>
+      <c r="B233" s="5" t="inlineStr">
+        <is>
+          <t>http://www.jweetmanlaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>Ball Law Offices, P.C.</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>http://dablaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="4" t="inlineStr">
+        <is>
+          <t>Madison Trademark Solutions</t>
+        </is>
+      </c>
+      <c r="B235" s="5" t="inlineStr">
+        <is>
+          <t>https://www.madisontrademarksolutions.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>Lemaire Patent Law Firm, PLLC</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lemairepatent.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="4" t="inlineStr">
+        <is>
+          <t>The Simon Law Firm, P.C.</t>
+        </is>
+      </c>
+      <c r="B237" s="5" t="inlineStr">
+        <is>
+          <t>https://simonlawpc.com/meet-our-attorneys/paul-j-tahan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>Husch Blackwell LLP</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>http://www.huschblackwell.com/bio.aspx?id=6600ef99-3d99-4953-bfcc-52a059ca52e4&amp;type=firm&amp;stype=a</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>Fortify Law LLC</t>
+        </is>
+      </c>
+      <c r="B239" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fortifylaw.com/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B225"/>
+  <autoFilter ref="A1:B239"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -3400,6 +3568,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B223" r:id="rId221"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B224" r:id="rId222"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B225" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B226" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B227" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B228" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B229" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B230" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B231" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B232" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B233" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B234" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B235" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B236" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B237" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B238" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B239" r:id="rId237"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToWidth="1"/>

</xml_diff>

<commit_message>
Continue collection: WI/UT/SC/OK page 2 batches
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cornell_ip_scraper/output/IP_Law_Firms.xlsx
+++ b/cornell_ip_scraper/output/IP_Law_Firms.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IP Law Firms" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$243</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'IP Law Firms'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B239"/>
+  <dimension ref="A1:B243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -3342,8 +3342,56 @@
         </is>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>Twisdale Law, PC</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>https://twisdalelaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="4" t="inlineStr">
+        <is>
+          <t>Sausser Summers, PC</t>
+        </is>
+      </c>
+      <c r="B241" s="5" t="inlineStr">
+        <is>
+          <t>https://onlinetrademarkattorneys.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>Clayton Howarth, P.C.</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>https://chcpat.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="4" t="inlineStr">
+        <is>
+          <t>Thrive IP</t>
+        </is>
+      </c>
+      <c r="B243" s="5" t="inlineStr">
+        <is>
+          <t>http://thrive-ip.com/about-us/bernard-s-ben-klosowski-jr-j-d/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B239"/>
+  <autoFilter ref="A1:B243"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -3582,6 +3630,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B237" r:id="rId235"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B238" r:id="rId236"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B239" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B240" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B241" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B242" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B243" r:id="rId241"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToWidth="1"/>

</xml_diff>

<commit_message>
Continue collection: CT/KY/LA + IN/IA/KS/AR batches
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cornell_ip_scraper/output/IP_Law_Firms.xlsx
+++ b/cornell_ip_scraper/output/IP_Law_Firms.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IP Law Firms" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$243</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IP Law Firms'!$A$1:$B$251</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'IP Law Firms'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B243"/>
+  <dimension ref="A1:B251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -553,7 +553,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CALHOUN LAW FIRM</t>
+          <t>Calhoun Law Firm</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -789,7 +789,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Martin, Pringle, Oliver, Wallace and Bauer, L.L.P.</t>
+          <t>Martin, Pringle, Oliver, Wallace &amp; Bauer, L.L.P.</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -3390,8 +3390,104 @@
         </is>
       </c>
     </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>McCarter &amp; English LLP</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>http://mccarter.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="4" t="inlineStr">
+        <is>
+          <t>The Gillispie Law Firm, P.S.C.</t>
+        </is>
+      </c>
+      <c r="B245" s="5" t="inlineStr">
+        <is>
+          <t>https://gillispielaw.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>Montague Law PLLC</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>https://wmlex.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="4" t="inlineStr">
+        <is>
+          <t>Kean Miller LLP</t>
+        </is>
+      </c>
+      <c r="B247" s="5" t="inlineStr">
+        <is>
+          <t>https://www.keanmiller.com/monica-j-manzella-cipp-us.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>Tong Law</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>http://www.tong-law.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="4" t="inlineStr">
+        <is>
+          <t>Hartman Law, P.C.</t>
+        </is>
+      </c>
+      <c r="B249" s="5" t="inlineStr">
+        <is>
+          <t>http://www.hplawoffices.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>Surge Business Law</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>https://surge.law/</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="4" t="inlineStr">
+        <is>
+          <t>Rock City Law, PLLC</t>
+        </is>
+      </c>
+      <c r="B251" s="5" t="inlineStr">
+        <is>
+          <t>https://www.rockcitylaw.com/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B243"/>
+  <autoFilter ref="A1:B251"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -3634,6 +3730,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B241" r:id="rId239"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B242" r:id="rId240"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B243" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B244" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B245" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B246" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B247" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B248" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B249" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B250" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B251" r:id="rId249"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToWidth="1"/>

</xml_diff>